<commit_message>
One voice at a time, and nothing repeats inside 90 seconds
- A clip may not repeat for at least 90 s, except greetings (meet, meet-reply and the shopkeepers' aao ji), which keep their own gap
- Street events (quarrels, crashes, colony fights, police chases, tipping autos) wait at least 90 s before the next one
- Only one recorded voice line plays at a time: a line that comes up while another is playing waits for it to finish (up to 6 s) instead of talking over it

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jnez1WfyLHPdoZrXbbanCH
</commit_message>
<xml_diff>
--- a/docs/voice-map.xlsx
+++ b/docs/voice-map.xlsx
@@ -543,7 +543,7 @@
         <v>12</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="J2" s="3" t="inlineStr"/>
     </row>
@@ -585,7 +585,7 @@
         <v>15</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="J3" s="3" t="inlineStr"/>
     </row>
@@ -627,7 +627,7 @@
         <v>15</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="J4" s="3" t="inlineStr"/>
     </row>
@@ -669,7 +669,7 @@
         <v>15</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="J5" s="3" t="inlineStr"/>
     </row>
@@ -1005,7 +1005,7 @@
         <v>15</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="J13" s="3" t="inlineStr"/>
     </row>
@@ -1425,7 +1425,7 @@
         <v>10</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="J23" s="3" t="inlineStr"/>
     </row>
@@ -1467,7 +1467,7 @@
         <v>10</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="J24" s="3" t="inlineStr"/>
     </row>
@@ -1509,7 +1509,7 @@
         <v>10</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="J25" s="3" t="inlineStr"/>
     </row>
@@ -1551,7 +1551,7 @@
         <v>10</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="J26" s="3" t="inlineStr"/>
     </row>
@@ -1593,7 +1593,7 @@
         <v>18</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="J27" s="3" t="inlineStr"/>
     </row>
@@ -1635,7 +1635,7 @@
         <v>18</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="J28" s="3" t="inlineStr"/>
     </row>
@@ -1677,7 +1677,7 @@
         <v>18</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="J29" s="3" t="inlineStr"/>
     </row>
@@ -1719,7 +1719,7 @@
         <v>20</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="J30" s="3" t="inlineStr"/>
     </row>
@@ -1761,7 +1761,7 @@
         <v>20</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="J31" s="3" t="inlineStr"/>
     </row>
@@ -1803,7 +1803,7 @@
         <v>20</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="J32" s="3" t="inlineStr"/>
     </row>
@@ -1845,7 +1845,7 @@
         <v>20</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="J33" s="3" t="inlineStr"/>
     </row>
@@ -1887,7 +1887,7 @@
         <v>22</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="J34" s="3" t="inlineStr"/>
     </row>
@@ -1929,7 +1929,7 @@
         <v>30</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>25</v>
+        <v>90</v>
       </c>
       <c r="J35" s="3" t="inlineStr"/>
     </row>
@@ -1971,7 +1971,7 @@
         <v>15</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="J36" s="3" t="inlineStr"/>
     </row>
@@ -2013,7 +2013,7 @@
         <v>45</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="J37" s="3" t="inlineStr"/>
     </row>
@@ -2055,7 +2055,7 @@
         <v>10</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="J38" s="3" t="inlineStr"/>
     </row>
@@ -2097,7 +2097,7 @@
         <v>10</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>8</v>
+        <v>90</v>
       </c>
       <c r="J39" s="3" t="inlineStr"/>
     </row>
@@ -2139,7 +2139,7 @@
         <v>10</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>8</v>
+        <v>90</v>
       </c>
       <c r="J40" s="3" t="inlineStr"/>
     </row>
@@ -2181,7 +2181,7 @@
         <v>12</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="J41" s="3" t="inlineStr"/>
     </row>
@@ -2223,7 +2223,7 @@
         <v>15</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="J42" s="3" t="inlineStr"/>
     </row>
@@ -2265,7 +2265,7 @@
         <v>15</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="J43" s="3" t="inlineStr"/>
     </row>
@@ -2307,7 +2307,7 @@
         <v>15</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="J44" s="3" t="inlineStr"/>
     </row>
@@ -2349,7 +2349,7 @@
         <v>15</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="J45" s="3" t="inlineStr"/>
     </row>
@@ -2391,7 +2391,7 @@
         <v>30</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>6</v>
+        <v>90</v>
       </c>
       <c r="J46" s="3" t="inlineStr"/>
     </row>
@@ -2433,7 +2433,7 @@
         <v>30</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>6</v>
+        <v>90</v>
       </c>
       <c r="J47" s="3" t="inlineStr"/>
     </row>
@@ -2475,7 +2475,7 @@
         <v>30</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>6</v>
+        <v>90</v>
       </c>
       <c r="J48" s="3" t="inlineStr"/>
     </row>
@@ -2517,7 +2517,7 @@
         <v>30</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>6</v>
+        <v>90</v>
       </c>
       <c r="J49" s="3" t="inlineStr"/>
     </row>
@@ -3495,7 +3495,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Min gap: seconds before the same clip can play again.</t>
+          <t>Min gap: seconds before the same clip can play again (never less than 90, except greetings).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Snake bikers, autos that skid and tip when hit, family-sized street fights, voices only from people you can see
- Snake bikers: now and then a biker turns up ahead and weaves about in front of you; hit him with your vehicle and the bike flies, he lands on the road, and you shout 'Oye! Aaya maza, sapp!' (new clip, desi Punjabi voice R). T panel can call one in
- Autos and e-rickshaws hit by any vehicle skid sideways and go over on their side; passengers spill and shout
- Street quarrels turn into family fights: two or three more on each side join once it gets physical; colony fights are three men and three women
- A resident's recorded line plays only if they are close (6 m) or in front of the camera with no wall in between, so no more aunty voices from nowhere

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jnez1WfyLHPdoZrXbbanCH
</commit_message>
<xml_diff>
--- a/docs/voice-map.xlsx
+++ b/docs/voice-map.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1351,17 +1351,17 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>player_ssa_f</t>
+          <t>player_sapp</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Sat Sri Akal ji! Tusi theek ho?</t>
+          <t>Oye! Aaya maza, sapp! Hahaha!</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Q — the player, female (Paaro)</t>
+          <t>R — the player's shout, desi Punjabi (Pind Waali)</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -1371,19 +1371,19 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>player-f</t>
+          <t>player</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>meet</t>
+          <t>snake-hit</t>
         </is>
       </c>
       <c r="H22" s="3" t="n">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>8</v>
+        <v>90</v>
       </c>
       <c r="J22" s="3" t="inlineStr"/>
     </row>
@@ -1393,17 +1393,17 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>gossip_a</t>
+          <t>player_ssa_f</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Pata ae? Gillan di nooh Canada chali gayi, te munda ethe hi reh gaya!</t>
+          <t>Sat Sri Akal ji! Tusi theek ho?</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>C — cheerful woman (Pammi's voice)</t>
+          <t>Q — the player, female (Paaro)</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -1413,19 +1413,19 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>any-woman</t>
+          <t>player-f</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>chat</t>
+          <t>meet</t>
         </is>
       </c>
       <c r="H23" s="3" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>90</v>
+        <v>8</v>
       </c>
       <c r="J23" s="3" t="inlineStr"/>
     </row>
@@ -1435,17 +1435,17 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>gossip_b</t>
+          <t>gossip_a</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Haaye! Main taan pehlan hi kehndi si!</t>
+          <t>Pata ae? Gillan di nooh Canada chali gayi, te munda ethe hi reh gaya!</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>B — dry woman (Gurnam's voice)</t>
+          <t>C — cheerful woman (Pammi's voice)</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -1477,17 +1477,17 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>chat_match</t>
+          <t>gossip_b</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Kal da match vekhya? Saadi team ne phir dil tod ditta!</t>
+          <t>Haaye! Main taan pehlan hi kehndi si!</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>F — loud man (angry neighbour voice)</t>
+          <t>B — dry woman (Gurnam's voice)</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -1497,7 +1497,7 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>any-man</t>
+          <t>any-woman</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -1519,17 +1519,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>chat_petrol</t>
+          <t>chat_match</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Petrol de bhaa vekh! Hun taan saikal hi changi ae.</t>
+          <t>Kal da match vekhya? Saadi team ne phir dil tod ditta!</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>G — old man (Ustad's voice)</t>
+          <t>F — loud man (angry neighbour voice)</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1539,7 +1539,7 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>any-man, any-elder</t>
+          <t>any-man</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -1561,17 +1561,17 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>call_sabzi</t>
+          <t>chat_petrol</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Aaloo lai lo, pyaaz lai lo! Taaze tamatar, sasti bhindi!</t>
+          <t>Petrol de bhaa vekh! Hun taan saikal hi changi ae.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>A — jolly man (Bhola's voice)</t>
+          <t>G — old man (Ustad's voice)</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1581,16 +1581,16 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>sabzi-wala</t>
+          <t>any-man, any-elder</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>street-call</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="H27" s="3" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>90</v>
@@ -1603,17 +1603,17 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>call_fruit</t>
+          <t>call_sabzi</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Kele lai lo, kinnow, mitthe ambh! Chakh ke dekho ji!</t>
+          <t>Aaloo lai lo, pyaaz lai lo! Taaze tamatar, sasti bhindi!</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>G — old man (Ustad's voice)</t>
+          <t>A — jolly man (Bhola's voice)</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>fruit-wala</t>
+          <t>sabzi-wala</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -1645,17 +1645,17 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>call_chaat</t>
+          <t>call_fruit</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Gol gappe! Teekhe vi, mitthe vi! Aao ji, aao!</t>
+          <t>Kele lai lo, kinnow, mitthe ambh! Chakh ke dekho ji!</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>A — jolly man (Bhola's voice)</t>
+          <t>G — old man (Ustad's voice)</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>chaat-wala</t>
+          <t>fruit-wala</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -1687,12 +1687,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>call_doodh</t>
+          <t>call_chaat</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Doodh waala aa gaya! Taaza doodh, bhenji!</t>
+          <t>Gol gappe! Teekhe vi, mitthe vi! Aao ji, aao!</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>doodh-wala</t>
+          <t>chaat-wala</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -1716,7 +1716,7 @@
         </is>
       </c>
       <c r="H30" s="3" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>90</v>
@@ -1729,17 +1729,17 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>call_kabadi</t>
+          <t>call_doodh</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Kabaadi waala! Purana loha, akhbaar, botlan — vech lo!</t>
+          <t>Doodh waala aa gaya! Taaza doodh, bhenji!</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>D — gruff man (police voice)</t>
+          <t>A — jolly man (Bhola's voice)</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>kabadi-wala</t>
+          <t>doodh-wala</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -1771,17 +1771,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>call_auto_gill</t>
+          <t>call_kabadi</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Gill, Gill, Gill! Gill Road, Gill! Aa jao, baith jao!</t>
+          <t>Kabaadi waala! Purana loha, akhbaar, botlan — vech lo!</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>E — young man (lafanga voice)</t>
+          <t>D — gruff man (police voice)</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>auto-wala</t>
+          <t>kabadi-wala</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -1813,17 +1813,17 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>call_auto_ludhiana</t>
+          <t>call_auto_gill</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Ludhiana, Ludhiana, Ludhiana! Bas do sawari hor, chalo chalo!</t>
+          <t>Gill, Gill, Gill! Gill Road, Gill! Aa jao, baith jao!</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>F — loud man (angry neighbour voice)</t>
+          <t>E — young man (lafanga voice)</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -1855,17 +1855,17 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>call_bus</t>
+          <t>call_auto_ludhiana</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Jalandhar, Phagwara, Ludhiana! Chhetti chadho, bus chalan lagi ae!</t>
+          <t>Ludhiana, Ludhiana, Ludhiana! Bas do sawari hor, chalo chalo!</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>D — gruff man (police voice)</t>
+          <t>F — loud man (angry neighbour voice)</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>bus-conductor, conductor</t>
+          <t>auto-wala</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -1884,7 +1884,7 @@
         </is>
       </c>
       <c r="H34" s="3" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>90</v>
@@ -1897,12 +1897,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>police_rukk</t>
+          <t>call_bus</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Oye! Rukk ja! Rukk ja, hero!</t>
+          <t>Jalandhar, Phagwara, Ludhiana! Chhetti chadho, bus chalan lagi ae!</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1917,16 +1917,16 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>police, police-bike</t>
+          <t>bus-conductor, conductor</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>police-chase, police-patrol</t>
+          <t>street-call</t>
         </is>
       </c>
       <c r="H35" s="3" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>90</v>
@@ -1939,12 +1939,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>police_chai</t>
+          <t>police_rukk</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Dekh puttar, case bada serious ae… chai-paani da intezaam karo, te gal khatam!</t>
+          <t>Oye! Rukk ja! Rukk ja, hero!</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1959,16 +1959,16 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>police, balwant</t>
+          <t>police, police-bike</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>police-bribe</t>
+          <t>police-chase, police-patrol</t>
         </is>
       </c>
       <c r="H36" s="3" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>90</v>
@@ -1981,12 +1981,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>police_gaddi_rok</t>
+          <t>police_chai</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Gaddi rok! Side te laa! Oye, sunda nahi?!</t>
+          <t>Dekh puttar, case bada serious ae… chai-paani da intezaam karo, te gal khatam!</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2001,16 +2001,16 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>police-jeep, police-bike</t>
+          <t>police, balwant</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>police-jeep, police-patrol</t>
+          <t>police-bribe</t>
         </is>
       </c>
       <c r="H37" s="3" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>90</v>
@@ -2023,17 +2023,17 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>lafanga_chai</t>
+          <t>police_gaddi_rok</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Ki dekh reha ae, hero? Saanu chai pila!</t>
+          <t>Gaddi rok! Side te laa! Oye, sunda nahi?!</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>E — young man (lafanga voice)</t>
+          <t>D — gruff man (police voice)</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2043,16 +2043,16 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>lafanga</t>
+          <t>police-jeep, police-bike</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>lafanga-taunt</t>
+          <t>police-jeep, police-patrol</t>
         </is>
       </c>
       <c r="H38" s="3" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>90</v>
@@ -2065,17 +2065,17 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>panga_bhen</t>
+          <t>lafanga_chai</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Teri bhen di! Mere naal panga?</t>
+          <t>Ki dekh reha ae, hero? Saanu chai pila!</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>? — made by the other session</t>
+          <t>E — young man (lafanga voice)</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
@@ -2085,12 +2085,12 @@
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>lafanga, any-man</t>
+          <t>lafanga</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>gang-fight, hit, fight-start</t>
+          <t>lafanga-taunt</t>
         </is>
       </c>
       <c r="H39" s="3" t="n">
@@ -2107,12 +2107,12 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>khad_dasda</t>
+          <t>panga_bhen</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Khad, tainu dasda haan!</t>
+          <t>Teri bhen di! Mere naal panga?</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2127,12 +2127,12 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>any-man, driver</t>
+          <t>lafanga, any-man</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>blame-both, road-rage, hit, fight-start</t>
+          <t>gang-fight, hit, fight-start</t>
         </is>
       </c>
       <c r="H40" s="3" t="n">
@@ -2149,12 +2149,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>ki_ho_gaya</t>
+          <t>khad_dasda</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Ki ho gaya ji? Ki ho gaya?</t>
+          <t>Khad, tainu dasda haan!</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2169,16 +2169,16 @@
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>onlooker</t>
+          <t>any-man, driver</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>quarrel-onlooker, fight-onlooker</t>
+          <t>blame-both, road-rage, hit, fight-start</t>
         </is>
       </c>
       <c r="H41" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>90</v>
@@ -2191,17 +2191,17 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>quarrel_kaun</t>
+          <t>ki_ho_gaya</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Tu jaanda nahi main kaun haan?!</t>
+          <t>Ki ho gaya ji? Ki ho gaya?</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>F — loud man (angry neighbour voice)</t>
+          <t>? — made by the other session</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2211,16 +2211,16 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>any-man</t>
+          <t>onlooker</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>quarrel-start, colony-fight-start</t>
+          <t>quarrel-onlooker, fight-onlooker</t>
         </is>
       </c>
       <c r="H42" s="3" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I42" s="3" t="n">
         <v>90</v>
@@ -2233,12 +2233,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>rage_andha</t>
+          <t>quarrel_kaun</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Oye! Andha ae? Meri gaddi da nuksaan kaun bharega?!</t>
+          <t>Tu jaanda nahi main kaun haan?!</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2253,12 +2253,12 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>driver</t>
+          <t>any-man</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>road-rage, crash-drivers</t>
+          <t>quarrel-start, colony-fight-start</t>
         </is>
       </c>
       <c r="H43" s="3" t="n">
@@ -2275,17 +2275,17 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>aunty_fight_1</t>
+          <t>rage_andha</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Ni kalmuhiye! Tera kutta roz mere boohe agge gand paunda ae!</t>
+          <t>Oye! Andha ae? Meri gaddi da nuksaan kaun bharega?!</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>C — cheerful woman (Pammi's voice)</t>
+          <t>F — loud man (angry neighbour voice)</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -2295,12 +2295,12 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>aunty</t>
+          <t>driver</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>aunty-quarrel-start, colony-fight-start</t>
+          <t>road-rage, crash-drivers</t>
         </is>
       </c>
       <c r="H44" s="3" t="n">
@@ -2317,17 +2317,17 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>aunty_fight_2</t>
+          <t>aunty_fight_1</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Chal ni chudail! Pehlan apne vehre di safai kar, phir gall kari!</t>
+          <t>Ni kalmuhiye! Tera kutta roz mere boohe agge gand paunda ae!</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>B — dry woman (Gurnam's voice)</t>
+          <t>C — cheerful woman (Pammi's voice)</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>aunty-quarrel-blows, colony-fight-blows</t>
+          <t>aunty-quarrel-start, colony-fight-start</t>
         </is>
       </c>
       <c r="H45" s="3" t="n">
@@ -2359,17 +2359,17 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>fuddu</t>
+          <t>aunty_fight_2</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Oye, fuddu ho gaya ae ki? Akkal ghaah charan gayi ae!</t>
+          <t>Chal ni chudail! Pehlan apne vehre di safai kar, phir gall kari!</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>E — young man (lafanga voice)</t>
+          <t>B — dry woman (Gurnam's voice)</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -2379,16 +2379,16 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>passenger</t>
+          <t>aunty</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>auto-tipped</t>
+          <t>aunty-quarrel-blows, colony-fight-blows</t>
         </is>
       </c>
       <c r="H46" s="3" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="I46" s="3" t="n">
         <v>90</v>
@@ -2401,17 +2401,17 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>bump_oye</t>
+          <t>fuddu</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Oye hoye! Dekh ke chala, hero! This is a bazaar, not a racetrack!</t>
+          <t>Oye, fuddu ho gaya ae ki? Akkal ghaah charan gayi ae!</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>B — dry woman (Gurnam's voice)</t>
+          <t>E — young man (lafanga voice)</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -2443,17 +2443,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>safari_kanjar</t>
+          <t>bump_oye</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Oye kanjar da puttar! Auto palat ditta! Hun paise nahi dene tere!</t>
+          <t>Oye hoye! Dekh ke chala, hero! This is a bazaar, not a racetrack!</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>F — loud man (angry neighbour voice)</t>
+          <t>B — dry woman (Gurnam's voice)</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -2485,17 +2485,17 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>sawari_lak</t>
+          <t>safari_kanjar</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Hai rabba! Mera lakk tutt gaya! Kithe dhyaan ae tera, fuddu?!</t>
+          <t>Oye kanjar da puttar! Auto palat ditta! Hun paise nahi dene tere!</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>C — cheerful woman (Pammi's voice)</t>
+          <t>F — loud man (angry neighbour voice)</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
@@ -2521,16 +2521,58 @@
       </c>
       <c r="J49" s="3" t="inlineStr"/>
     </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>sawari_lak</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Hai rabba! Mera lakk tutt gaya! Kithe dhyaan ae tera, fuddu?!</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>C — cheerful woman (Pammi's voice)</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>passenger</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>auto-tipped</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I50" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J50" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="E2:E49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E2:E50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F2:F50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>Codes!$A$2:$A$44</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>Codes!$C$2:$C$34</formula1>
+    <dataValidation sqref="G2:G50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>Codes!$C$2:$C$35</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3311,8 +3353,16 @@
           <t>a bus conductor</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>snake-hit</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>you knock a zig-zag snake biker off his bike</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">

</xml_diff>

<commit_message>
Player's line to an old uncle in a fight
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017nSM5vQNCHuCUh6sR8Nzza
</commit_message>
<xml_diff>
--- a/docs/voice-map.xlsx
+++ b/docs/voice-map.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1435,17 +1435,17 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>gossip_a</t>
+          <t>player_uncle_gitte</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Pata ae? Gillan di nooh Canada chali gayi, te munda ethe hi reh gaya!</t>
+          <t>Oh uncle ji, tuhada dimaag thode gitteyan vich hai ki?</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>C — cheerful woman (Pammi's voice)</t>
+          <t>P — the player, male (Deepak)</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -1455,16 +1455,16 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>any-woman</t>
+          <t>player</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>chat</t>
+          <t>fight-elder</t>
         </is>
       </c>
       <c r="H24" s="3" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>90</v>
@@ -1477,17 +1477,17 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>gossip_b</t>
+          <t>gossip_a</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Haaye! Main taan pehlan hi kehndi si!</t>
+          <t>Pata ae? Gillan di nooh Canada chali gayi, te munda ethe hi reh gaya!</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>B — dry woman (Gurnam's voice)</t>
+          <t>C — cheerful woman (Pammi's voice)</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -1519,17 +1519,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>chat_match</t>
+          <t>gossip_b</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Kal da match vekhya? Saadi team ne phir dil tod ditta!</t>
+          <t>Haaye! Main taan pehlan hi kehndi si!</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>F — loud man (angry neighbour voice)</t>
+          <t>B — dry woman (Gurnam's voice)</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1539,7 +1539,7 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>any-man</t>
+          <t>any-woman</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -1561,17 +1561,17 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>chat_petrol</t>
+          <t>chat_match</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Petrol de bhaa vekh! Hun taan saikal hi changi ae.</t>
+          <t>Kal da match vekhya? Saadi team ne phir dil tod ditta!</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>G — old man (Ustad's voice)</t>
+          <t>F — loud man (angry neighbour voice)</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>any-man, any-elder</t>
+          <t>any-man</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -1603,17 +1603,17 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>call_sabzi</t>
+          <t>chat_petrol</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Aaloo lai lo, pyaaz lai lo! Taaze tamatar, sasti bhindi!</t>
+          <t>Petrol de bhaa vekh! Hun taan saikal hi changi ae.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>A — jolly man (Bhola's voice)</t>
+          <t>G — old man (Ustad's voice)</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -1623,16 +1623,16 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>sabzi-wala</t>
+          <t>any-man, any-elder</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>street-call</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="H28" s="3" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>90</v>
@@ -1645,17 +1645,17 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>call_fruit</t>
+          <t>call_sabzi</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Kele lai lo, kinnow, mitthe ambh! Chakh ke dekho ji!</t>
+          <t>Aaloo lai lo, pyaaz lai lo! Taaze tamatar, sasti bhindi!</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>G — old man (Ustad's voice)</t>
+          <t>A — jolly man (Bhola's voice)</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>fruit-wala</t>
+          <t>sabzi-wala</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -1687,17 +1687,17 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>call_chaat</t>
+          <t>call_fruit</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Gol gappe! Teekhe vi, mitthe vi! Aao ji, aao!</t>
+          <t>Kele lai lo, kinnow, mitthe ambh! Chakh ke dekho ji!</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>A — jolly man (Bhola's voice)</t>
+          <t>G — old man (Ustad's voice)</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>chaat-wala</t>
+          <t>fruit-wala</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -1729,12 +1729,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>call_doodh</t>
+          <t>call_chaat</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Doodh waala aa gaya! Taaza doodh, bhenji!</t>
+          <t>Gol gappe! Teekhe vi, mitthe vi! Aao ji, aao!</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>doodh-wala</t>
+          <t>chaat-wala</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -1758,7 +1758,7 @@
         </is>
       </c>
       <c r="H31" s="3" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>90</v>
@@ -1771,17 +1771,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>call_kabadi</t>
+          <t>call_doodh</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Kabaadi waala! Purana loha, akhbaar, botlan — vech lo!</t>
+          <t>Doodh waala aa gaya! Taaza doodh, bhenji!</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>D — gruff man (police voice)</t>
+          <t>A — jolly man (Bhola's voice)</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>kabadi-wala</t>
+          <t>doodh-wala</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -1813,17 +1813,17 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>call_auto_gill</t>
+          <t>call_kabadi</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Gill, Gill, Gill! Gill Road, Gill! Aa jao, baith jao!</t>
+          <t>Kabaadi waala! Purana loha, akhbaar, botlan — vech lo!</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>E — young man (lafanga voice)</t>
+          <t>D — gruff man (police voice)</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>auto-wala</t>
+          <t>kabadi-wala</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -1855,17 +1855,17 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>call_auto_ludhiana</t>
+          <t>call_auto_gill</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Ludhiana, Ludhiana, Ludhiana! Bas do sawari hor, chalo chalo!</t>
+          <t>Gill, Gill, Gill! Gill Road, Gill! Aa jao, baith jao!</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>F — loud man (angry neighbour voice)</t>
+          <t>E — young man (lafanga voice)</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -1897,17 +1897,17 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>call_bus</t>
+          <t>call_auto_ludhiana</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Jalandhar, Phagwara, Ludhiana! Chhetti chadho, bus chalan lagi ae!</t>
+          <t>Ludhiana, Ludhiana, Ludhiana! Bas do sawari hor, chalo chalo!</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>D — gruff man (police voice)</t>
+          <t>F — loud man (angry neighbour voice)</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -1917,7 +1917,7 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>bus-conductor, conductor</t>
+          <t>auto-wala</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -1926,7 +1926,7 @@
         </is>
       </c>
       <c r="H35" s="3" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>90</v>
@@ -1939,12 +1939,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>police_rukk</t>
+          <t>call_bus</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Oye! Rukk ja! Rukk ja, hero!</t>
+          <t>Jalandhar, Phagwara, Ludhiana! Chhetti chadho, bus chalan lagi ae!</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1959,16 +1959,16 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>police, police-bike</t>
+          <t>bus-conductor, conductor</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>police-chase, police-patrol</t>
+          <t>street-call</t>
         </is>
       </c>
       <c r="H36" s="3" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>90</v>
@@ -1981,12 +1981,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>police_chai</t>
+          <t>police_rukk</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Dekh puttar, case bada serious ae… chai-paani da intezaam karo, te gal khatam!</t>
+          <t>Oye! Rukk ja! Rukk ja, hero!</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2001,16 +2001,16 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>police, balwant</t>
+          <t>police, police-bike</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>police-bribe</t>
+          <t>police-chase, police-patrol</t>
         </is>
       </c>
       <c r="H37" s="3" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>90</v>
@@ -2023,12 +2023,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>police_gaddi_rok</t>
+          <t>police_chai</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Gaddi rok! Side te laa! Oye, sunda nahi?!</t>
+          <t>Dekh puttar, case bada serious ae… chai-paani da intezaam karo, te gal khatam!</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2043,16 +2043,16 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>police-jeep, police-bike</t>
+          <t>police, balwant</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>police-jeep, police-patrol</t>
+          <t>police-bribe</t>
         </is>
       </c>
       <c r="H38" s="3" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>90</v>
@@ -2065,17 +2065,17 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>lafanga_chai</t>
+          <t>police_gaddi_rok</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Ki dekh reha ae, hero? Saanu chai pila!</t>
+          <t>Gaddi rok! Side te laa! Oye, sunda nahi?!</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>E — young man (lafanga voice)</t>
+          <t>D — gruff man (police voice)</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
@@ -2085,16 +2085,16 @@
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>lafanga</t>
+          <t>police-jeep, police-bike</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>lafanga-taunt</t>
+          <t>police-jeep, police-patrol</t>
         </is>
       </c>
       <c r="H39" s="3" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>90</v>
@@ -2107,17 +2107,17 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>panga_bhen</t>
+          <t>lafanga_chai</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Teri bhen di! Mere naal panga?</t>
+          <t>Ki dekh reha ae, hero? Saanu chai pila!</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>? — made by the other session</t>
+          <t>E — young man (lafanga voice)</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -2127,12 +2127,12 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>lafanga, any-man</t>
+          <t>lafanga</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>gang-fight, hit, fight-start</t>
+          <t>lafanga-taunt</t>
         </is>
       </c>
       <c r="H40" s="3" t="n">
@@ -2149,12 +2149,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>khad_dasda</t>
+          <t>panga_bhen</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Khad, tainu dasda haan!</t>
+          <t>Teri bhen di! Mere naal panga?</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2169,12 +2169,12 @@
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>any-man, driver</t>
+          <t>lafanga, any-man</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>blame-both, road-rage, hit, fight-start</t>
+          <t>gang-fight, hit, fight-start</t>
         </is>
       </c>
       <c r="H41" s="3" t="n">
@@ -2191,12 +2191,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>ki_ho_gaya</t>
+          <t>khad_dasda</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Ki ho gaya ji? Ki ho gaya?</t>
+          <t>Khad, tainu dasda haan!</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2211,16 +2211,16 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>onlooker</t>
+          <t>any-man, driver</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>quarrel-onlooker, fight-onlooker</t>
+          <t>blame-both, road-rage, hit, fight-start</t>
         </is>
       </c>
       <c r="H42" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I42" s="3" t="n">
         <v>90</v>
@@ -2233,17 +2233,17 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>quarrel_kaun</t>
+          <t>ki_ho_gaya</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Tu jaanda nahi main kaun haan?!</t>
+          <t>Ki ho gaya ji? Ki ho gaya?</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>F — loud man (angry neighbour voice)</t>
+          <t>? — made by the other session</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
@@ -2253,16 +2253,16 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>any-man</t>
+          <t>onlooker</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>quarrel-start, colony-fight-start</t>
+          <t>quarrel-onlooker, fight-onlooker</t>
         </is>
       </c>
       <c r="H43" s="3" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I43" s="3" t="n">
         <v>90</v>
@@ -2275,12 +2275,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>rage_andha</t>
+          <t>quarrel_kaun</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Oye! Andha ae? Meri gaddi da nuksaan kaun bharega?!</t>
+          <t>Tu jaanda nahi main kaun haan?!</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2295,12 +2295,12 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>driver</t>
+          <t>any-man</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>road-rage, crash-drivers</t>
+          <t>quarrel-start, colony-fight-start</t>
         </is>
       </c>
       <c r="H44" s="3" t="n">
@@ -2317,17 +2317,17 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>aunty_fight_1</t>
+          <t>rage_andha</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Ni kalmuhiye! Tera kutta roz mere boohe agge gand paunda ae!</t>
+          <t>Oye! Andha ae? Meri gaddi da nuksaan kaun bharega?!</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>C — cheerful woman (Pammi's voice)</t>
+          <t>F — loud man (angry neighbour voice)</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
@@ -2337,12 +2337,12 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>aunty</t>
+          <t>driver</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>aunty-quarrel-start, colony-fight-start</t>
+          <t>road-rage, crash-drivers</t>
         </is>
       </c>
       <c r="H45" s="3" t="n">
@@ -2359,17 +2359,17 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>aunty_fight_2</t>
+          <t>aunty_fight_1</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Chal ni chudail! Pehlan apne vehre di safai kar, phir gall kari!</t>
+          <t>Ni kalmuhiye! Tera kutta roz mere boohe agge gand paunda ae!</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>B — dry woman (Gurnam's voice)</t>
+          <t>C — cheerful woman (Pammi's voice)</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>aunty-quarrel-blows, colony-fight-blows</t>
+          <t>aunty-quarrel-start, colony-fight-start</t>
         </is>
       </c>
       <c r="H46" s="3" t="n">
@@ -2401,17 +2401,17 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>fuddu</t>
+          <t>aunty_fight_2</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Oye, fuddu ho gaya ae ki? Akkal ghaah charan gayi ae!</t>
+          <t>Chal ni chudail! Pehlan apne vehre di safai kar, phir gall kari!</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>E — young man (lafanga voice)</t>
+          <t>B — dry woman (Gurnam's voice)</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -2421,16 +2421,16 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>passenger</t>
+          <t>aunty</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>auto-tipped</t>
+          <t>aunty-quarrel-blows, colony-fight-blows</t>
         </is>
       </c>
       <c r="H47" s="3" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="I47" s="3" t="n">
         <v>90</v>
@@ -2443,17 +2443,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>bump_oye</t>
+          <t>fuddu</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Oye hoye! Dekh ke chala, hero! This is a bazaar, not a racetrack!</t>
+          <t>Oye, fuddu ho gaya ae ki? Akkal ghaah charan gayi ae!</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>B — dry woman (Gurnam's voice)</t>
+          <t>E — young man (lafanga voice)</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -2485,17 +2485,17 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>safari_kanjar</t>
+          <t>bump_oye</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Oye kanjar da puttar! Auto palat ditta! Hun paise nahi dene tere!</t>
+          <t>Oye hoye! Dekh ke chala, hero! This is a bazaar, not a racetrack!</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>F — loud man (angry neighbour voice)</t>
+          <t>B — dry woman (Gurnam's voice)</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
@@ -2527,17 +2527,17 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>sawari_lak</t>
+          <t>safari_kanjar</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Hai rabba! Mera lakk tutt gaya! Kithe dhyaan ae tera, fuddu?!</t>
+          <t>Oye kanjar da puttar! Auto palat ditta! Hun paise nahi dene tere!</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>C — cheerful woman (Pammi's voice)</t>
+          <t>F — loud man (angry neighbour voice)</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
@@ -2563,15 +2563,57 @@
       </c>
       <c r="J50" s="3" t="inlineStr"/>
     </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>sawari_lak</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Hai rabba! Mera lakk tutt gaya! Kithe dhyaan ae tera, fuddu?!</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>C — cheerful woman (Pammi's voice)</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>passenger</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>auto-tipped</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I51" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J51" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="E2:E50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E2:E51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F2:F51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>Codes!$A$2:$A$44</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>Codes!$C$2:$C$35</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Rain and flood reactions: people react as it pours and curse the choked drains
Eight new voice lines (aunties caught in the rain, uncles on the MLA and the
drains, autowalas refusing the flooded bazaar) are on the voice map switched
off until they are recorded; until then the words show as speech bubbles.
New when codes rain-start and flood; tool tools/raintalk.mjs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLbA8kD2DzB3Kx6vn5ahzP
</commit_message>
<xml_diff>
--- a/docs/voice-map.xlsx
+++ b/docs/voice-map.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1477,12 +1477,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>gossip_a</t>
+          <t>rain_suit</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Pata ae? Gillan di nooh Canada chali gayi, te munda ethe hi reh gaya!</t>
+          <t>Haaye mera suit! Chhatri vi ghar reh gayi, hun taan poori bhijj gayi!</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -1502,14 +1502,14 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>chat</t>
+          <t>rain-start</t>
         </is>
       </c>
       <c r="H25" s="3" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="J25" s="3" t="inlineStr"/>
     </row>
@@ -1519,12 +1519,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>gossip_b</t>
+          <t>rain_kapde</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Haaye! Main taan pehlan hi kehndi si!</t>
+          <t>Ni Simran, chhatt ton kapde laah chheti! Meeh aa gaya!</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -1544,14 +1544,14 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>chat</t>
+          <t>rain-start</t>
         </is>
       </c>
       <c r="H26" s="3" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="J26" s="3" t="inlineStr"/>
     </row>
@@ -1561,39 +1561,39 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>chat_match</t>
+          <t>rain_chhatri_aunty</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Kal da match vekhya? Saadi team ne phir dil tod ditta!</t>
+          <t>Hatt ke chal puttar, chhatri naal akh na kadh dayin kise di!</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>F — loud man (angry neighbour voice)</t>
+          <t>B — dry woman (Gurnam's voice)</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>any-man</t>
+          <t>any-woman, any-elder</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>chat</t>
+          <t>rain-start, flood</t>
         </is>
       </c>
       <c r="H27" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="J27" s="3" t="inlineStr"/>
     </row>
@@ -1603,39 +1603,39 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>chat_petrol</t>
+          <t>rain_pakode</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Petrol de bhaa vekh! Hun taan saikal hi changi ae.</t>
+          <t>Meeh vich taan garam pakode te chah hi bandi ae!</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>G — old man (Ustad's voice)</t>
+          <t>A — jolly man (Bhola's voice)</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>any-man, any-elder</t>
+          <t>any-man</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>chat</t>
+          <t>rain-start</t>
         </is>
       </c>
       <c r="H28" s="3" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="J28" s="3" t="inlineStr"/>
     </row>
@@ -1645,39 +1645,39 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>call_sabzi</t>
+          <t>flood_mla</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Aaloo lai lo, pyaaz lai lo! Taaze tamatar, sasti bhindi!</t>
+          <t>Har saal eho haal! MLA sahib vote lain aunde ne, naali saaf karaun koi nahi aunda!</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>A — jolly man (Bhola's voice)</t>
+          <t>G — old man (Ustad's voice)</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>sabzi-wala</t>
+          <t>any-elder, any-man</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>street-call</t>
+          <t>flood</t>
         </is>
       </c>
       <c r="H29" s="3" t="n">
         <v>18</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="J29" s="3" t="inlineStr"/>
     </row>
@@ -1687,39 +1687,39 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>call_fruit</t>
+          <t>flood_naali</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Kele lai lo, kinnow, mitthe ambh! Chakh ke dekho ji!</t>
+          <t>Naaliyan band ne, saara paani gali vich! Committee waale so rahe ne!</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>G — old man (Ustad's voice)</t>
+          <t>F — loud man (angry neighbour voice)</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>fruit-wala</t>
+          <t>any-man</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>street-call</t>
+          <t>flood</t>
         </is>
       </c>
       <c r="H30" s="3" t="n">
         <v>18</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="J30" s="3" t="inlineStr"/>
     </row>
@@ -1729,39 +1729,39 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>call_chaat</t>
+          <t>flood_auto_engine</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Gol gappe! Teekhe vi, mitthe vi! Aao ji, aao!</t>
+          <t>Paani bahut ae ji, engine band ho jaau! Kiraya doona lagga!</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>A — jolly man (Bhola's voice)</t>
+          <t>E — young man (lafanga voice)</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>chaat-wala</t>
+          <t>auto-wala</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>street-call</t>
+          <t>flood</t>
         </is>
       </c>
       <c r="H31" s="3" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="J31" s="3" t="inlineStr"/>
     </row>
@@ -1771,39 +1771,39 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>call_doodh</t>
+          <t>flood_auto_kishti</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Doodh waala aa gaya! Taaza doodh, bhenji!</t>
+          <t>Na ji, Dal Bazaar nahi jaana! Othe taan kishti chahidi ae!</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>A — jolly man (Bhola's voice)</t>
+          <t>F — loud man (angry neighbour voice)</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>doodh-wala</t>
+          <t>auto-wala</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>street-call</t>
+          <t>flood</t>
         </is>
       </c>
       <c r="H32" s="3" t="n">
         <v>20</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="J32" s="3" t="inlineStr"/>
     </row>
@@ -1813,17 +1813,17 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>call_kabadi</t>
+          <t>gossip_a</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Kabaadi waala! Purana loha, akhbaar, botlan — vech lo!</t>
+          <t>Pata ae? Gillan di nooh Canada chali gayi, te munda ethe hi reh gaya!</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>D — gruff man (police voice)</t>
+          <t>C — cheerful woman (Pammi's voice)</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -1833,16 +1833,16 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>kabadi-wala</t>
+          <t>any-woman</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>street-call</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="H33" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>90</v>
@@ -1855,17 +1855,17 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>call_auto_gill</t>
+          <t>gossip_b</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Gill, Gill, Gill! Gill Road, Gill! Aa jao, baith jao!</t>
+          <t>Haaye! Main taan pehlan hi kehndi si!</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>E — young man (lafanga voice)</t>
+          <t>B — dry woman (Gurnam's voice)</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -1875,16 +1875,16 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>auto-wala</t>
+          <t>any-woman</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>street-call</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="H34" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>90</v>
@@ -1897,12 +1897,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>call_auto_ludhiana</t>
+          <t>chat_match</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Ludhiana, Ludhiana, Ludhiana! Bas do sawari hor, chalo chalo!</t>
+          <t>Kal da match vekhya? Saadi team ne phir dil tod ditta!</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1917,16 +1917,16 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>auto-wala</t>
+          <t>any-man</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>street-call</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="H35" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>90</v>
@@ -1939,17 +1939,17 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>call_bus</t>
+          <t>chat_petrol</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Jalandhar, Phagwara, Ludhiana! Chhetti chadho, bus chalan lagi ae!</t>
+          <t>Petrol de bhaa vekh! Hun taan saikal hi changi ae.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>D — gruff man (police voice)</t>
+          <t>G — old man (Ustad's voice)</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -1959,16 +1959,16 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>bus-conductor, conductor</t>
+          <t>any-man, any-elder</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>street-call</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="H36" s="3" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>90</v>
@@ -1981,17 +1981,17 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>police_rukk</t>
+          <t>call_sabzi</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Oye! Rukk ja! Rukk ja, hero!</t>
+          <t>Aaloo lai lo, pyaaz lai lo! Taaze tamatar, sasti bhindi!</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>D — gruff man (police voice)</t>
+          <t>A — jolly man (Bhola's voice)</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
@@ -2001,16 +2001,16 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>police, police-bike</t>
+          <t>sabzi-wala</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>police-chase, police-patrol</t>
+          <t>street-call</t>
         </is>
       </c>
       <c r="H37" s="3" t="n">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>90</v>
@@ -2023,17 +2023,17 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>police_chai</t>
+          <t>call_fruit</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Dekh puttar, case bada serious ae… chai-paani da intezaam karo, te gal khatam!</t>
+          <t>Kele lai lo, kinnow, mitthe ambh! Chakh ke dekho ji!</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>D — gruff man (police voice)</t>
+          <t>G — old man (Ustad's voice)</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2043,16 +2043,16 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>police, balwant</t>
+          <t>fruit-wala</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>police-bribe</t>
+          <t>street-call</t>
         </is>
       </c>
       <c r="H38" s="3" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>90</v>
@@ -2065,17 +2065,17 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>police_gaddi_rok</t>
+          <t>call_chaat</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Gaddi rok! Side te laa! Oye, sunda nahi?!</t>
+          <t>Gol gappe! Teekhe vi, mitthe vi! Aao ji, aao!</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>D — gruff man (police voice)</t>
+          <t>A — jolly man (Bhola's voice)</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
@@ -2085,16 +2085,16 @@
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>police-jeep, police-bike</t>
+          <t>chaat-wala</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>police-jeep, police-patrol</t>
+          <t>street-call</t>
         </is>
       </c>
       <c r="H39" s="3" t="n">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>90</v>
@@ -2107,17 +2107,17 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>lafanga_chai</t>
+          <t>call_doodh</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Ki dekh reha ae, hero? Saanu chai pila!</t>
+          <t>Doodh waala aa gaya! Taaza doodh, bhenji!</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>E — young man (lafanga voice)</t>
+          <t>A — jolly man (Bhola's voice)</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -2127,16 +2127,16 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>lafanga</t>
+          <t>doodh-wala</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>lafanga-taunt</t>
+          <t>street-call</t>
         </is>
       </c>
       <c r="H40" s="3" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>90</v>
@@ -2149,17 +2149,17 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>panga_bhen</t>
+          <t>call_kabadi</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Teri bhen di! Mere naal panga?</t>
+          <t>Kabaadi waala! Purana loha, akhbaar, botlan — vech lo!</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>? — made by the other session</t>
+          <t>D — gruff man (police voice)</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
@@ -2169,16 +2169,16 @@
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>lafanga, any-man</t>
+          <t>kabadi-wala</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>gang-fight, hit, fight-start</t>
+          <t>street-call</t>
         </is>
       </c>
       <c r="H41" s="3" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>90</v>
@@ -2191,17 +2191,17 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>khad_dasda</t>
+          <t>call_auto_gill</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Khad, tainu dasda haan!</t>
+          <t>Gill, Gill, Gill! Gill Road, Gill! Aa jao, baith jao!</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>? — made by the other session</t>
+          <t>E — young man (lafanga voice)</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2211,16 +2211,16 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>any-man, driver</t>
+          <t>auto-wala</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>blame-both, road-rage, hit, fight-start</t>
+          <t>street-call</t>
         </is>
       </c>
       <c r="H42" s="3" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="I42" s="3" t="n">
         <v>90</v>
@@ -2233,17 +2233,17 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>ki_ho_gaya</t>
+          <t>call_auto_ludhiana</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Ki ho gaya ji? Ki ho gaya?</t>
+          <t>Ludhiana, Ludhiana, Ludhiana! Bas do sawari hor, chalo chalo!</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>? — made by the other session</t>
+          <t>F — loud man (angry neighbour voice)</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
@@ -2253,16 +2253,16 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>onlooker</t>
+          <t>auto-wala</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>quarrel-onlooker, fight-onlooker</t>
+          <t>street-call</t>
         </is>
       </c>
       <c r="H43" s="3" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="I43" s="3" t="n">
         <v>90</v>
@@ -2275,17 +2275,17 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>quarrel_kaun</t>
+          <t>call_bus</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Tu jaanda nahi main kaun haan?!</t>
+          <t>Jalandhar, Phagwara, Ludhiana! Chhetti chadho, bus chalan lagi ae!</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>F — loud man (angry neighbour voice)</t>
+          <t>D — gruff man (police voice)</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -2295,16 +2295,16 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>any-man</t>
+          <t>bus-conductor, conductor</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>quarrel-start, colony-fight-start</t>
+          <t>street-call</t>
         </is>
       </c>
       <c r="H44" s="3" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="I44" s="3" t="n">
         <v>90</v>
@@ -2317,17 +2317,17 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>rage_andha</t>
+          <t>police_rukk</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Oye! Andha ae? Meri gaddi da nuksaan kaun bharega?!</t>
+          <t>Oye! Rukk ja! Rukk ja, hero!</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>F — loud man (angry neighbour voice)</t>
+          <t>D — gruff man (police voice)</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
@@ -2337,16 +2337,16 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>driver</t>
+          <t>police, police-bike</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>road-rage, crash-drivers</t>
+          <t>police-chase, police-patrol</t>
         </is>
       </c>
       <c r="H45" s="3" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="I45" s="3" t="n">
         <v>90</v>
@@ -2359,17 +2359,17 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>aunty_fight_1</t>
+          <t>police_chai</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Ni kalmuhiye! Tera kutta roz mere boohe agge gand paunda ae!</t>
+          <t>Dekh puttar, case bada serious ae… chai-paani da intezaam karo, te gal khatam!</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>C — cheerful woman (Pammi's voice)</t>
+          <t>D — gruff man (police voice)</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -2379,12 +2379,12 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>aunty</t>
+          <t>police, balwant</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>aunty-quarrel-start, colony-fight-start</t>
+          <t>police-bribe</t>
         </is>
       </c>
       <c r="H46" s="3" t="n">
@@ -2401,17 +2401,17 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>aunty_fight_2</t>
+          <t>police_gaddi_rok</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Chal ni chudail! Pehlan apne vehre di safai kar, phir gall kari!</t>
+          <t>Gaddi rok! Side te laa! Oye, sunda nahi?!</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>B — dry woman (Gurnam's voice)</t>
+          <t>D — gruff man (police voice)</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -2421,16 +2421,16 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>aunty</t>
+          <t>police-jeep, police-bike</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>aunty-quarrel-blows, colony-fight-blows</t>
+          <t>police-jeep, police-patrol</t>
         </is>
       </c>
       <c r="H47" s="3" t="n">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="I47" s="3" t="n">
         <v>90</v>
@@ -2443,12 +2443,12 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>fuddu</t>
+          <t>lafanga_chai</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Oye, fuddu ho gaya ae ki? Akkal ghaah charan gayi ae!</t>
+          <t>Ki dekh reha ae, hero? Saanu chai pila!</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2463,16 +2463,16 @@
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>passenger</t>
+          <t>lafanga</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>auto-tipped</t>
+          <t>lafanga-taunt</t>
         </is>
       </c>
       <c r="H48" s="3" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="I48" s="3" t="n">
         <v>90</v>
@@ -2485,17 +2485,17 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>bump_oye</t>
+          <t>panga_bhen</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Oye hoye! Dekh ke chala, hero! This is a bazaar, not a racetrack!</t>
+          <t>Teri bhen di! Mere naal panga?</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>B — dry woman (Gurnam's voice)</t>
+          <t>? — made by the other session</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
@@ -2505,16 +2505,16 @@
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>passenger</t>
+          <t>lafanga, any-man</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>auto-tipped</t>
+          <t>gang-fight, hit, fight-start</t>
         </is>
       </c>
       <c r="H49" s="3" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="I49" s="3" t="n">
         <v>90</v>
@@ -2527,17 +2527,17 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>safari_kanjar</t>
+          <t>khad_dasda</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Oye kanjar da puttar! Auto palat ditta! Hun paise nahi dene tere!</t>
+          <t>Khad, tainu dasda haan!</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>F — loud man (angry neighbour voice)</t>
+          <t>? — made by the other session</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
@@ -2547,16 +2547,16 @@
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>passenger</t>
+          <t>any-man, driver</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>auto-tipped</t>
+          <t>blame-both, road-rage, hit, fight-start</t>
         </is>
       </c>
       <c r="H50" s="3" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="I50" s="3" t="n">
         <v>90</v>
@@ -2569,17 +2569,17 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>sawari_lak</t>
+          <t>ki_ho_gaya</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Hai rabba! Mera lakk tutt gaya! Kithe dhyaan ae tera, fuddu?!</t>
+          <t>Ki ho gaya ji? Ki ho gaya?</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>C — cheerful woman (Pammi's voice)</t>
+          <t>? — made by the other session</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
@@ -2589,32 +2589,368 @@
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>passenger</t>
+          <t>onlooker</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>auto-tipped</t>
+          <t>quarrel-onlooker, fight-onlooker</t>
         </is>
       </c>
       <c r="H51" s="3" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="I51" s="3" t="n">
         <v>90</v>
       </c>
       <c r="J51" s="3" t="inlineStr"/>
     </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>quarrel_kaun</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Tu jaanda nahi main kaun haan?!</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>F — loud man (angry neighbour voice)</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>any-man</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>quarrel-start, colony-fight-start</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I52" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>rage_andha</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Oye! Andha ae? Meri gaddi da nuksaan kaun bharega?!</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>F — loud man (angry neighbour voice)</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>driver</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>road-rage, crash-drivers</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I53" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>aunty_fight_1</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Ni kalmuhiye! Tera kutta roz mere boohe agge gand paunda ae!</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>C — cheerful woman (Pammi's voice)</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>aunty</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>aunty-quarrel-start, colony-fight-start</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I54" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>aunty_fight_2</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Chal ni chudail! Pehlan apne vehre di safai kar, phir gall kari!</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>B — dry woman (Gurnam's voice)</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>aunty</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>aunty-quarrel-blows, colony-fight-blows</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I55" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>fuddu</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Oye, fuddu ho gaya ae ki? Akkal ghaah charan gayi ae!</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>E — young man (lafanga voice)</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>passenger</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>auto-tipped</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I56" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J56" s="3" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>bump_oye</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Oye hoye! Dekh ke chala, hero! This is a bazaar, not a racetrack!</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>B — dry woman (Gurnam's voice)</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>passenger</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>auto-tipped</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I57" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>safari_kanjar</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Oye kanjar da puttar! Auto palat ditta! Hun paise nahi dene tere!</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>F — loud man (angry neighbour voice)</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>passenger</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>auto-tipped</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I58" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J58" s="3" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>sawari_lak</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Hai rabba! Mera lakk tutt gaya! Kithe dhyaan ae tera, fuddu?!</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>C — cheerful woman (Pammi's voice)</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>passenger</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>auto-tipped</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I59" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J59" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="E2:E51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E2:E59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F2:F59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>Codes!$A$2:$A$44</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>Codes!$C$2:$C$35</formula1>
+    <dataValidation sqref="G2:G59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>Codes!$C$2:$C$38</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3417,8 +3753,16 @@
           <t>sabzi seller</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>fight-elder</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>you square up to an old uncle</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3431,8 +3775,16 @@
           <t>fruit seller</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>rain-start</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>it starts to pour: someone near you reacts</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3445,8 +3797,16 @@
           <t>gol-gappe / chaat seller</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>flood</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>the galis are flooded: someone near you complains</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">

</xml_diff>

<commit_message>
Voice: record the eight rain and flood lines (ElevenLabs, Punjabi voices), switch them on
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EKfKCZd8Db7yDFAHyPwGvs
</commit_message>
<xml_diff>
--- a/docs/voice-map.xlsx
+++ b/docs/voice-map.xlsx
@@ -1492,7 +1492,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">

</xml_diff>

<commit_message>
50 recorded voice lines for doorbell, power cuts, rail gates, pump, bank, post, signals and friends; the game calendar with seasonal fields
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UtxJKyY1yRfzeoJ6kY8TJE
</commit_message>
<xml_diff>
--- a/docs/voice-map.xlsx
+++ b/docs/voice-map.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J109"/>
+  <dimension ref="A1:J159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -5041,16 +5041,2116 @@
       </c>
       <c r="J109" s="3" t="inlineStr"/>
     </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>v2_bell_01</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Kaun ae, ji? Ki gal ae?</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>T — aunty, middle-aged woman (Ritu Rathore)</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>any-woman, any-elder</t>
+        </is>
+      </c>
+      <c r="G110" s="3" t="inlineStr">
+        <is>
+          <t>doorbell-stranger</t>
+        </is>
+      </c>
+      <c r="H110" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I110" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J110" s="3" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>v2_bell_02</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Haanji, ki chahida? Ruko, aa rahi haan!</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>C — cheerful woman (Pammi's voice)</t>
+        </is>
+      </c>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F111" s="3" t="inlineStr">
+        <is>
+          <t>any-woman</t>
+        </is>
+      </c>
+      <c r="G111" s="3" t="inlineStr">
+        <is>
+          <t>doorbell-stranger</t>
+        </is>
+      </c>
+      <c r="H111" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I111" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J111" s="3" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>v2_bell_03</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>Sadde ghar kuj nahi chahida, ji. Shukriya!</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>T — aunty, middle-aged woman (Ritu Rathore)</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>any-woman, any-elder</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="inlineStr">
+        <is>
+          <t>doorbell-stranger</t>
+        </is>
+      </c>
+      <c r="H112" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I112" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J112" s="3" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>v2_bell_04</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>Haanji paaji, ki hukam ae?</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>A — jolly man (Bhola's voice)</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>any-man</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
+          <t>doorbell-stranger</t>
+        </is>
+      </c>
+      <c r="H113" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I113" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J113" s="3" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>v2_bell_05</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>Kiss nu milna ae, puttar? Andar aa ja!</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>S — Punjabi shopkeeper man (Saurav)</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>any-man, any-elder</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="inlineStr">
+        <is>
+          <t>doorbell-stranger</t>
+        </is>
+      </c>
+      <c r="H114" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I114" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J114" s="3" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>v2_bell_06</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>Oye kaun ae? Zara ruk, buddhe nu uthan de!</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>G — old man (Ustad's voice)</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F115" s="3" t="inlineStr">
+        <is>
+          <t>any-man, any-elder</t>
+        </is>
+      </c>
+      <c r="G115" s="3" t="inlineStr">
+        <is>
+          <t>doorbell-stranger</t>
+        </is>
+      </c>
+      <c r="H115" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I115" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J115" s="3" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>v2_bell_07</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>Aa gaya puttar? Waheguru, bahut din baad!</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>G — old man (Ustad's voice)</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>any-man, any-elder</t>
+        </is>
+      </c>
+      <c r="G116" s="3" t="inlineStr">
+        <is>
+          <t>doorbell-family</t>
+        </is>
+      </c>
+      <c r="H116" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I116" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J116" s="3" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>v2_bell_08</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>Hai, galat ghar aa gaye ho shayad, paaji.</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>B — dry woman (Gurnam's voice)</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F117" s="3" t="inlineStr">
+        <is>
+          <t>any-woman, any-elder</t>
+        </is>
+      </c>
+      <c r="G117" s="3" t="inlineStr">
+        <is>
+          <t>doorbell-stranger</t>
+        </is>
+      </c>
+      <c r="H117" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I117" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J117" s="3" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>v2_gate_01</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>Oye, tu aa gaya! Andar aa, chah pee ke jaayi!</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>A — jolly man (Bhola's voice)</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="inlineStr">
+        <is>
+          <t>any-man</t>
+        </is>
+      </c>
+      <c r="G118" s="3" t="inlineStr">
+        <is>
+          <t>doorbell-family</t>
+        </is>
+      </c>
+      <c r="H118" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I118" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J118" s="3" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>v2_gate_02</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>Haye puttar, bahut vadhia kita jo aa gaya! Mummy ghar ae.</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>G — old man (Ustad's voice)</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="inlineStr">
+        <is>
+          <t>any-man, any-elder</t>
+        </is>
+      </c>
+      <c r="G119" s="3" t="inlineStr">
+        <is>
+          <t>doorbell-family</t>
+        </is>
+      </c>
+      <c r="H119" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I119" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J119" s="3" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>v2_gate_03</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>Sat Sri Akal ji! Aaj bahut dina baad chakkar laaya ae!</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>T — aunty, middle-aged woman (Ritu Rathore)</t>
+        </is>
+      </c>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F120" s="3" t="inlineStr">
+        <is>
+          <t>any-woman, any-elder</t>
+        </is>
+      </c>
+      <c r="G120" s="3" t="inlineStr">
+        <is>
+          <t>doorbell-family</t>
+        </is>
+      </c>
+      <c r="H120" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I120" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J120" s="3" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>v2_gate_04</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>Aaja aaja, gate khula ae! Pehchaan liya si tenu!</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>C — cheerful woman (Pammi's voice)</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="inlineStr">
+        <is>
+          <t>any-woman</t>
+        </is>
+      </c>
+      <c r="G121" s="3" t="inlineStr">
+        <is>
+          <t>doorbell-family</t>
+        </is>
+      </c>
+      <c r="H121" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I121" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J121" s="3" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>v2_night_01</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>Eni raat nu kaun ae? Subah aana, puttar!</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>G — old man (Ustad's voice)</t>
+        </is>
+      </c>
+      <c r="E122" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F122" s="3" t="inlineStr">
+        <is>
+          <t>any-elder</t>
+        </is>
+      </c>
+      <c r="G122" s="3" t="inlineStr">
+        <is>
+          <t>doorbell-night</t>
+        </is>
+      </c>
+      <c r="H122" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I122" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J122" s="3" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>v2_night_02</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>Raat bahut ho gayi, kal aao ji!</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>T — aunty, middle-aged woman (Ritu Rathore)</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>any-woman</t>
+        </is>
+      </c>
+      <c r="G123" s="3" t="inlineStr">
+        <is>
+          <t>doorbell-night</t>
+        </is>
+      </c>
+      <c r="H123" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I123" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J123" s="3" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>v2_night_03</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>Oye! Sab sau gaye ne, subah gal karange!</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>F — loud man (angry neighbour voice)</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F124" s="3" t="inlineStr">
+        <is>
+          <t>any-man</t>
+        </is>
+      </c>
+      <c r="G124" s="3" t="inlineStr">
+        <is>
+          <t>doorbell-night</t>
+        </is>
+      </c>
+      <c r="H124" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I124" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J124" s="3" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>v2_siesta_01</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>Oh ho, dupehar nu sau rahe haan! Baad vich aana.</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>B — dry woman (Gurnam's voice)</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F125" s="3" t="inlineStr">
+        <is>
+          <t>any-woman</t>
+        </is>
+      </c>
+      <c r="G125" s="3" t="inlineStr">
+        <is>
+          <t>doorbell-siesta</t>
+        </is>
+      </c>
+      <c r="H125" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I125" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J125" s="3" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>v2_siesta_02</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>Hai rabba, ajj vi araam nahi! Kaun ae?</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>T — aunty, middle-aged woman (Ritu Rathore)</t>
+        </is>
+      </c>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F126" s="3" t="inlineStr">
+        <is>
+          <t>any-woman</t>
+        </is>
+      </c>
+      <c r="G126" s="3" t="inlineStr">
+        <is>
+          <t>doorbell-siesta</t>
+        </is>
+      </c>
+      <c r="H126" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I126" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J126" s="3" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>v2_cut_01</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>Hai rabba, bijli phir gayi! Inverter laga lo!</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>C — cheerful woman (Pammi's voice)</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F127" s="3" t="inlineStr">
+        <is>
+          <t>any-woman</t>
+        </is>
+      </c>
+      <c r="G127" s="3" t="inlineStr">
+        <is>
+          <t>power-cut</t>
+        </is>
+      </c>
+      <c r="H127" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I127" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J127" s="3" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>v2_cut_02</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>PSPCL walon ne phir kamaal kar ditta!</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>A — jolly man (Bhola's voice)</t>
+        </is>
+      </c>
+      <c r="E128" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F128" s="3" t="inlineStr">
+        <is>
+          <t>any-man</t>
+        </is>
+      </c>
+      <c r="G128" s="3" t="inlineStr">
+        <is>
+          <t>power-cut</t>
+        </is>
+      </c>
+      <c r="H128" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I128" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J128" s="3" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>v2_cut_03</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>Roz roz light cut, hun taan hadd ho gayi!</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>F — loud man (angry neighbour voice)</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F129" s="3" t="inlineStr">
+        <is>
+          <t>any-man</t>
+        </is>
+      </c>
+      <c r="G129" s="3" t="inlineStr">
+        <is>
+          <t>power-cut</t>
+        </is>
+      </c>
+      <c r="H129" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I129" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J129" s="3" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>v2_cut_04</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>Mobile da charge vi nahi hoya si, haaye!</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>T — aunty, middle-aged woman (Ritu Rathore)</t>
+        </is>
+      </c>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F130" s="3" t="inlineStr">
+        <is>
+          <t>any-woman</t>
+        </is>
+      </c>
+      <c r="G130" s="3" t="inlineStr">
+        <is>
+          <t>power-cut</t>
+        </is>
+      </c>
+      <c r="H130" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I130" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J130" s="3" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>v2_cut_05</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>Saade vele taan lalten hundi si, koi fikar nahi!</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>G — old man (Ustad's voice)</t>
+        </is>
+      </c>
+      <c r="E131" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F131" s="3" t="inlineStr">
+        <is>
+          <t>any-elder</t>
+        </is>
+      </c>
+      <c r="G131" s="3" t="inlineStr">
+        <is>
+          <t>power-cut</t>
+        </is>
+      </c>
+      <c r="H131" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I131" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J131" s="3" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>v2_back_01</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>Aa gayi bijli! Shukar ae Waheguru da!</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>E — young man (lafanga voice)</t>
+        </is>
+      </c>
+      <c r="E132" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F132" s="3" t="inlineStr">
+        <is>
+          <t>any-man, young-man</t>
+        </is>
+      </c>
+      <c r="G132" s="3" t="inlineStr">
+        <is>
+          <t>power-back</t>
+        </is>
+      </c>
+      <c r="H132" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I132" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J132" s="3" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>v2_back_02</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>Light aa gayi! Chalo, tv lagao!</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>C — cheerful woman (Pammi's voice)</t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="inlineStr">
+        <is>
+          <t>any-woman</t>
+        </is>
+      </c>
+      <c r="G133" s="3" t="inlineStr">
+        <is>
+          <t>power-back</t>
+        </is>
+      </c>
+      <c r="H133" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I133" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J133" s="3" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>v2_rail_01</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>Phatak band ho gaya! Hun das minute!</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>F — loud man (angry neighbour voice)</t>
+        </is>
+      </c>
+      <c r="E134" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F134" s="3" t="inlineStr">
+        <is>
+          <t>any-man</t>
+        </is>
+      </c>
+      <c r="G134" s="3" t="inlineStr">
+        <is>
+          <t>rail-gate</t>
+        </is>
+      </c>
+      <c r="H134" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="I134" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J134" s="3" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>v2_rail_02</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>Train aa rahi ae, ruko ji, ruko!</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>A — jolly man (Bhola's voice)</t>
+        </is>
+      </c>
+      <c r="E135" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F135" s="3" t="inlineStr">
+        <is>
+          <t>any-man</t>
+        </is>
+      </c>
+      <c r="G135" s="3" t="inlineStr">
+        <is>
+          <t>rail-gate</t>
+        </is>
+      </c>
+      <c r="H135" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="I135" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J135" s="3" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>v2_rail_03</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>Eh phatak taan roz hi band rehnda ae!</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>T — aunty, middle-aged woman (Ritu Rathore)</t>
+        </is>
+      </c>
+      <c r="E136" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F136" s="3" t="inlineStr">
+        <is>
+          <t>any-woman</t>
+        </is>
+      </c>
+      <c r="G136" s="3" t="inlineStr">
+        <is>
+          <t>rail-gate</t>
+        </is>
+      </c>
+      <c r="H136" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="I136" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J136" s="3" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>v2_rail_04</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>Saade vele railway line te koi gaddi nahi aundi si.</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>G — old man (Ustad's voice)</t>
+        </is>
+      </c>
+      <c r="E137" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F137" s="3" t="inlineStr">
+        <is>
+          <t>any-elder</t>
+        </is>
+      </c>
+      <c r="G137" s="3" t="inlineStr">
+        <is>
+          <t>rail-gate</t>
+        </is>
+      </c>
+      <c r="H137" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="I137" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J137" s="3" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>v2_pump_01</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>Full kar ditta, paaji! Safar mubarak!</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>A — jolly man (Bhola's voice)</t>
+        </is>
+      </c>
+      <c r="E138" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F138" s="3" t="inlineStr">
+        <is>
+          <t>pumpwala</t>
+        </is>
+      </c>
+      <c r="G138" s="3" t="inlineStr">
+        <is>
+          <t>pump-done</t>
+        </is>
+      </c>
+      <c r="H138" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I138" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J138" s="3" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>v2_pump_02</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>Petrol, diesel, hawa; sab kujh milda ethe!</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>S — Punjabi shopkeeper man (Saurav)</t>
+        </is>
+      </c>
+      <c r="E139" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F139" s="3" t="inlineStr">
+        <is>
+          <t>pumpwala</t>
+        </is>
+      </c>
+      <c r="G139" s="3" t="inlineStr">
+        <is>
+          <t>pump-arrive</t>
+        </is>
+      </c>
+      <c r="H139" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I139" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J139" s="3" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>v2_pump_03</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>Meter dekh lo ji, zero ton shuru kitta si!</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>F — loud man (angry neighbour voice)</t>
+        </is>
+      </c>
+      <c r="E140" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F140" s="3" t="inlineStr">
+        <is>
+          <t>pumpwala</t>
+        </is>
+      </c>
+      <c r="G140" s="3" t="inlineStr">
+        <is>
+          <t>pump-done</t>
+        </is>
+      </c>
+      <c r="H140" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I140" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J140" s="3" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>v2_fuel_p1</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>Oye! Tank khaali ho gaya, hun dhakka lagauna painda!</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>P — the player, male (Deepak)</t>
+        </is>
+      </c>
+      <c r="E141" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F141" s="3" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="G141" s="3" t="inlineStr">
+        <is>
+          <t>fuel-out</t>
+        </is>
+      </c>
+      <c r="H141" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I141" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J141" s="3" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>v2_fuel_p2</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>Hai rabba, petrol khatam! Pump kithe ae?</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>P — the player, male (Deepak)</t>
+        </is>
+      </c>
+      <c r="E142" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F142" s="3" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="G142" s="3" t="inlineStr">
+        <is>
+          <t>fuel-out</t>
+        </is>
+      </c>
+      <c r="H142" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I142" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J142" s="3" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>v2_fuel_q1</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>Hai rabba, tank khaali! Hun ki karaan?</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>Q — the player, female (Paaro)</t>
+        </is>
+      </c>
+      <c r="E143" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F143" s="3" t="inlineStr">
+        <is>
+          <t>player-f</t>
+        </is>
+      </c>
+      <c r="G143" s="3" t="inlineStr">
+        <is>
+          <t>fuel-out</t>
+        </is>
+      </c>
+      <c r="H143" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I143" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J143" s="3" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>v2_fuel_q2</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>Oho, petrol khatam! Koi dhakka laga do!</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>Q — the player, female (Paaro)</t>
+        </is>
+      </c>
+      <c r="E144" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F144" s="3" t="inlineStr">
+        <is>
+          <t>player-f</t>
+        </is>
+      </c>
+      <c r="G144" s="3" t="inlineStr">
+        <is>
+          <t>fuel-out</t>
+        </is>
+      </c>
+      <c r="H144" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I144" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J144" s="3" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>v2_bank_01</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>Aao ji, Panj Aab Bank vich swagat ae. Ki seva karaan?</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>S — Punjabi shopkeeper man (Saurav)</t>
+        </is>
+      </c>
+      <c r="E145" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F145" s="3" t="inlineStr">
+        <is>
+          <t>clerk_bank</t>
+        </is>
+      </c>
+      <c r="G145" s="3" t="inlineStr">
+        <is>
+          <t>bank-welcome</t>
+        </is>
+      </c>
+      <c r="H145" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I145" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J145" s="3" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>v2_bank_02</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>Paise bank vich rakho, jeb vich nahi, puttar.</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>S — Punjabi shopkeeper man (Saurav)</t>
+        </is>
+      </c>
+      <c r="E146" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F146" s="3" t="inlineStr">
+        <is>
+          <t>clerk_bank</t>
+        </is>
+      </c>
+      <c r="G146" s="3" t="inlineStr">
+        <is>
+          <t>bank-advice</t>
+        </is>
+      </c>
+      <c r="H146" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I146" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J146" s="3" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>v2_post_01</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>Aao ji, ajj di dak aayi ae tuhadi.</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>G — old man (Ustad's voice)</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F147" s="3" t="inlineStr">
+        <is>
+          <t>clerk_post</t>
+        </is>
+      </c>
+      <c r="G147" s="3" t="inlineStr">
+        <is>
+          <t>post-welcome</t>
+        </is>
+      </c>
+      <c r="H147" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I147" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J147" s="3" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>v2_post_02</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>Chitthi aayi ae, Canada ton! Eh lo ji.</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>G — old man (Ustad's voice)</t>
+        </is>
+      </c>
+      <c r="E148" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F148" s="3" t="inlineStr">
+        <is>
+          <t>clerk_post</t>
+        </is>
+      </c>
+      <c r="G148" s="3" t="inlineStr">
+        <is>
+          <t>post-welcome</t>
+        </is>
+      </c>
+      <c r="H148" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I148" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="J148" s="3" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>v2_signal_01</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>Oye lal batti si! Akhan band ne ki?!</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>F — loud man (angry neighbour voice)</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>any-man</t>
+        </is>
+      </c>
+      <c r="G149" s="3" t="inlineStr">
+        <is>
+          <t>signal-jump</t>
+        </is>
+      </c>
+      <c r="H149" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="I149" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J149" s="3" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>v2_signal_02</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>Veere, signal tod ke kitthe chaleya?</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>E — young man (lafanga voice)</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F150" s="3" t="inlineStr">
+        <is>
+          <t>any-man, young-man</t>
+        </is>
+      </c>
+      <c r="G150" s="3" t="inlineStr">
+        <is>
+          <t>signal-jump</t>
+        </is>
+      </c>
+      <c r="H150" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="I150" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J150" s="3" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>v2_signal_03</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>Hai, hun taan thok dinda ae! Dhyaan naal!</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>B — dry woman (Gurnam's voice)</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F151" s="3" t="inlineStr">
+        <is>
+          <t>any-woman</t>
+        </is>
+      </c>
+      <c r="G151" s="3" t="inlineStr">
+        <is>
+          <t>signal-jump</t>
+        </is>
+      </c>
+      <c r="H151" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="I151" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J151" s="3" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>v2_friend_01</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>Oye sher! Kidhar gayab ho gaya si, yaar?</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>E — young man (lafanga voice)</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F152" s="3" t="inlineStr">
+        <is>
+          <t>any-man, young-man</t>
+        </is>
+      </c>
+      <c r="G152" s="3" t="inlineStr">
+        <is>
+          <t>meet-friend</t>
+        </is>
+      </c>
+      <c r="H152" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I152" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J152" s="3" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>v2_friend_02</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>Chal, chai pee lainde haan, sab kujh daseyo!</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>F — loud man (angry neighbour voice)</t>
+        </is>
+      </c>
+      <c r="E153" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F153" s="3" t="inlineStr">
+        <is>
+          <t>any-man</t>
+        </is>
+      </c>
+      <c r="G153" s="3" t="inlineStr">
+        <is>
+          <t>meet-friend</t>
+        </is>
+      </c>
+      <c r="H153" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I153" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J153" s="3" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>v2_friend_03</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>Yaar, tu taan hun bada banda ban gaya ae!</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>A — jolly man (Bhola's voice)</t>
+        </is>
+      </c>
+      <c r="E154" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F154" s="3" t="inlineStr">
+        <is>
+          <t>any-man</t>
+        </is>
+      </c>
+      <c r="G154" s="3" t="inlineStr">
+        <is>
+          <t>meet-friend</t>
+        </is>
+      </c>
+      <c r="H154" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I154" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J154" s="3" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>v2_friend_04</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>Tere bina taan gali sooni lagdi si, veere!</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>B — dry woman (Gurnam's voice)</t>
+        </is>
+      </c>
+      <c r="E155" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F155" s="3" t="inlineStr">
+        <is>
+          <t>any-woman</t>
+        </is>
+      </c>
+      <c r="G155" s="3" t="inlineStr">
+        <is>
+          <t>meet-friend</t>
+        </is>
+      </c>
+      <c r="H155" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I155" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J155" s="3" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>v2_meet_01</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>Ae ki, tu Gurnam da munda nahi? Kinna vadda ho gaya!</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>S — Punjabi shopkeeper man (Saurav)</t>
+        </is>
+      </c>
+      <c r="E156" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F156" s="3" t="inlineStr">
+        <is>
+          <t>any-man</t>
+        </is>
+      </c>
+      <c r="G156" s="3" t="inlineStr">
+        <is>
+          <t>meet-reply</t>
+        </is>
+      </c>
+      <c r="H156" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I156" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J156" s="3" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>v2_meet_02</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>Nava gaddi? Waah, chhakka maar ditta tu taan!</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>D — gruff man (police voice)</t>
+        </is>
+      </c>
+      <c r="E157" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F157" s="3" t="inlineStr">
+        <is>
+          <t>any-man, young-man</t>
+        </is>
+      </c>
+      <c r="G157" s="3" t="inlineStr">
+        <is>
+          <t>vehicle-admire</t>
+        </is>
+      </c>
+      <c r="H157" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I157" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="J157" s="3" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>v2_meet_03</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>Bhenji, tuhada puttar taan bade kamaal da ae!</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>Q — the player, female (Paaro)</t>
+        </is>
+      </c>
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F158" s="3" t="inlineStr">
+        <is>
+          <t>any-woman</t>
+        </is>
+      </c>
+      <c r="G158" s="3" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+      <c r="H158" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I158" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J158" s="3" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>v2_meet_04</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>Sat Sri Akal, ji! Kaim ho? Pind vich sab changa?</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>P — the player, male (Deepak)</t>
+        </is>
+      </c>
+      <c r="E159" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F159" s="3" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="G159" s="3" t="inlineStr">
+        <is>
+          <t>meet</t>
+        </is>
+      </c>
+      <c r="H159" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I159" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="J159" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="E2:E109" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E2:E159" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F109" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>Codes!$A$2:$A$44</formula1>
+    <dataValidation sqref="F2:F159" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>Codes!$A$2:$A$46</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G109" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>Codes!$C$2:$C$38</formula1>
+    <dataValidation sqref="G2:G159" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>Codes!$C$2:$C$54</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5063,7 +7163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5537,12 +7637,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>any-man</t>
+          <t>clerk_bank</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>any adult man</t>
+          <t>Anand sahib — bank manager</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -5559,12 +7659,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>young-man</t>
+          <t>clerk_post</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>a young man</t>
+          <t>Dhillon ji — postmaster</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -5581,12 +7681,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>any-woman</t>
+          <t>any-man</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>any adult woman</t>
+          <t>any adult man</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -5603,12 +7703,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>any-elder</t>
+          <t>young-man</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>any old man or woman</t>
+          <t>a young man</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -5625,12 +7725,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>shopkeeper-man</t>
+          <t>any-woman</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>a male shopkeeper</t>
+          <t>any adult woman</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -5647,12 +7747,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>shopkeeper-woman</t>
+          <t>any-elder</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>a female shopkeeper</t>
+          <t>any old man or woman</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -5669,12 +7769,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>aunty</t>
+          <t>shopkeeper-man</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>an aunty (in an aunty quarrel)</t>
+          <t>a male shopkeeper</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -5691,12 +7791,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>police</t>
+          <t>shopkeeper-woman</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>any constable / havaldar</t>
+          <t>a female shopkeeper</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -5713,12 +7813,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>police-jeep</t>
+          <t>aunty</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>the police jeep's loudspeaker</t>
+          <t>an aunty (in an aunty quarrel)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -5735,12 +7835,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>police-bike</t>
+          <t>police</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>a police motorbike rider</t>
+          <t>any constable / havaldar</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -5757,12 +7857,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>police-jeep</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>you (the player character)</t>
+          <t>the police jeep's loudspeaker</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -5779,12 +7879,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>lafanga</t>
+          <t>police-bike</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>a lafanga (street tough)</t>
+          <t>a police motorbike rider</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -5801,12 +7901,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>auto-wala</t>
+          <t>player</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>an auto-wala at a stand</t>
+          <t>you (the player character)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -5823,12 +7923,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>bus-conductor</t>
+          <t>lafanga</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>a bus conductor</t>
+          <t>a lafanga (street tough)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -5845,12 +7945,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>sabzi-wala</t>
+          <t>auto-wala</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>sabzi seller</t>
+          <t>an auto-wala at a stand</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -5867,12 +7967,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>fruit-wala</t>
+          <t>bus-conductor</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>fruit seller</t>
+          <t>a bus conductor</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -5889,12 +7989,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>chaat-wala</t>
+          <t>sabzi-wala</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>gol-gappe / chaat seller</t>
+          <t>sabzi seller</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -5911,86 +8011,290 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>doodh-wala</t>
+          <t>fruit-wala</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>milkman</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
+          <t>fruit seller</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>doorbell-stranger</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>you ring a stranger's bell and they answer at the gate</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>kabadi-wala</t>
+          <t>chaat-wala</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>scrap buyer</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
+          <t>gol-gappe / chaat seller</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>doorbell-family</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>you ring the bell of a family that knows yours</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>driver</t>
+          <t>doodh-wala</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>a driver you bumped</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
+          <t>milkman</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>doorbell-night</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>you ring a bell at night: a voice from a window</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>passenger</t>
+          <t>kabadi-wala</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>an auto passenger</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
+          <t>scrap buyer</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>doorbell-siesta</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>you ring a bell in the afternoon rest hour</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>onlooker</t>
+          <t>driver</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>a bystander watching a fight</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
+          <t>a driver you bumped</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>power-cut</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>the light goes: someone near you complains</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>passenger</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>an auto passenger</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>power-back</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>the light comes back: someone near you cheers</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>onlooker</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>a bystander watching a fight</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>rail-gate</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>the level-crossing gates close: someone near you complains</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>anyone</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>anyone at all</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>pump-arrive</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>you pull up at the petrol pump</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>pump-done</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>the tank is full</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>fuel-out</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>your tank runs dry</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>bank-welcome</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>you step up to the bank counter</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>bank-advice</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>you finish at the bank counter</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>post-welcome</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>you collect the post</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>signal-jump</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>you cross a junction against a red light: a bystander shouts</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>meet-friend</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>a friend answers your greeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>vehicle-admire</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>you get off a vehicle and someone near you admires it</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>